<commit_message>
custom model instead of linear in filter 6
</commit_message>
<xml_diff>
--- a/src/models/jupyter_files/common/info.xlsx
+++ b/src/models/jupyter_files/common/info.xlsx
@@ -8,19 +8,20 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="U:\ML_project\Bargh_ML\src\models\jupyter_files\common\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA875B0F-6C0F-48B4-A40E-89998659CDF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D07BAB8-0145-40A4-B364-6AF8C3FB6252}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="246" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="548" uniqueCount="53">
   <si>
     <t>name</t>
   </si>
@@ -124,9 +125,6 @@
     <t>detail</t>
   </si>
   <si>
-    <t>نبود temp_sens</t>
-  </si>
-  <si>
     <t>نقطه پرت داشت. اصلاح شد</t>
   </si>
   <si>
@@ -136,25 +134,52 @@
     <t>خط درست برازش شده ولی مطلوب نیست</t>
   </si>
   <si>
-    <t>اختلاف تولید در فصل سرما و تابستان باعث دو ترند در نمودار شده است</t>
-  </si>
-  <si>
-    <t>خط خوبی پیدا نشد. وجود داده پرت</t>
-  </si>
-  <si>
-    <t>ترند مکس با ترند میانگین یکی نبود</t>
-  </si>
-  <si>
     <t>داده‌ کم داریم</t>
   </si>
   <si>
     <t xml:space="preserve">B </t>
   </si>
   <si>
-    <t>exception می‌خوریم</t>
-  </si>
-  <si>
-    <t>به دل ننشست</t>
+    <t>همه حالت زینی شکل دارند و داده ها به هیچ وجه مطلوب نیست</t>
+  </si>
+  <si>
+    <t>حالت زینی شکل دارد</t>
+  </si>
+  <si>
+    <t>حالت زینی شکل دارد با temp_sens ولی با temperature خطی است</t>
+  </si>
+  <si>
+    <t>نبود temp_sens ـ- با temperature مشکل داده حل شد اما شکل خط نبود</t>
+  </si>
+  <si>
+    <t>temp_sens exception می‌خوریم اما با temperature شبیه  B می‌شود</t>
+  </si>
+  <si>
+    <t>اختلاف تولید در فصل سرما و تابستان باعث دو ترند در نمودار شده است - با temperature خوبه</t>
+  </si>
+  <si>
+    <t>خط خوبی پیدا نشد. وجود داده پرت - با temperature خوبه</t>
+  </si>
+  <si>
+    <t>به دل ننشست  - با temperature خوبه</t>
+  </si>
+  <si>
+    <t>ترند مکس با ترند میانگین یکی نبود -  با temperature خوبه</t>
+  </si>
+  <si>
+    <t>پرسش ۱</t>
+  </si>
+  <si>
+    <t>پرسش ۲</t>
+  </si>
+  <si>
+    <t>توصیف ۳</t>
+  </si>
+  <si>
+    <t>نه دو ترند دارد و یک خط</t>
+  </si>
+  <si>
+    <t>نمودار بی‌نظیر برای جدا شدن تاریخی</t>
   </si>
 </sst>
 </file>
@@ -210,10 +235,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -235,14 +263,33 @@
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{107A0CE5-8594-4619-91D2-B18464F48ACD}" name="Table1" displayName="Table1" ref="A1:D1048575" totalsRowShown="0">
   <autoFilter ref="A1:D1048575" xr:uid="{107A0CE5-8594-4619-91D2-B18464F48ACD}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D77">
-    <sortCondition ref="A1:A1048575"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D73">
+    <sortCondition ref="C1:C1048575"/>
   </sortState>
   <tableColumns count="4">
     <tableColumn id="2" xr3:uid="{42EA0A3D-0E11-4815-B659-3174AC86B68D}" name="name"/>
     <tableColumn id="3" xr3:uid="{400B851D-9539-4C1A-8177-93CB13B5EC72}" name="code"/>
     <tableColumn id="4" xr3:uid="{2AECFC46-919C-4A2E-BE6E-CB71F46CD1E6}" name="state"/>
     <tableColumn id="5" xr3:uid="{81060D6B-0411-4341-8021-D6876724D0C1}" name="detail"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{5907EC46-01FE-4BC8-93C8-E815CF551A07}" name="Table13" displayName="Table13" ref="A1:G1048575" totalsRowShown="0">
+  <autoFilter ref="A1:G1048575" xr:uid="{5907EC46-01FE-4BC8-93C8-E815CF551A07}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D73">
+    <sortCondition ref="C1:C1048575"/>
+  </sortState>
+  <tableColumns count="7">
+    <tableColumn id="2" xr3:uid="{02A9F4C6-3B73-4F51-9BB9-F251DD06EB60}" name="name"/>
+    <tableColumn id="3" xr3:uid="{12D6691A-B6DD-4E14-A4E0-186CA553C3BD}" name="code"/>
+    <tableColumn id="4" xr3:uid="{F0D0C0C2-1492-4AC9-BD7A-23B893C14659}" name="state"/>
+    <tableColumn id="5" xr3:uid="{AD89D0A4-90A9-4C73-BA49-17E4A6BBAD89}" name="detail"/>
+    <tableColumn id="7" xr3:uid="{4A3BE490-65FE-4529-AC07-4D135D71F124}" name="پرسش ۱"/>
+    <tableColumn id="6" xr3:uid="{490A7444-AC63-409F-9C80-F65FEEACDAC5}" name="پرسش ۲"/>
+    <tableColumn id="1" xr3:uid="{E485F360-6048-4496-A234-8334C714B2AC}" name="توصیف ۳"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -539,7 +586,7 @@
     <col min="1" max="1" width="18.88671875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="9.5546875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="7.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="48.77734375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="66.109375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="15.6640625" customWidth="1"/>
     <col min="7" max="7" width="34.21875" bestFit="1" customWidth="1"/>
   </cols>
@@ -620,10 +667,10 @@
         <v>27</v>
       </c>
       <c r="F5" t="s">
+        <v>35</v>
+      </c>
+      <c r="G5" t="s">
         <v>36</v>
-      </c>
-      <c r="G5" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
@@ -661,13 +708,13 @@
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="B9" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C9" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="D9" t="s">
         <v>34</v>
@@ -675,58 +722,46 @@
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C10" t="s">
-        <v>29</v>
-      </c>
-      <c r="D10" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="B11" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C11" t="s">
-        <v>29</v>
-      </c>
-      <c r="D11" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="B12" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C12" t="s">
-        <v>29</v>
-      </c>
-      <c r="D12" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="B13" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C13" t="s">
-        <v>29</v>
-      </c>
-      <c r="D13" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.3">
@@ -734,18 +769,15 @@
         <v>9</v>
       </c>
       <c r="B14" t="s">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="C14" t="s">
         <v>27</v>
-      </c>
-      <c r="D14" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B15" t="s">
         <v>4</v>
@@ -756,10 +788,10 @@
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B16" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C16" t="s">
         <v>27</v>
@@ -767,10 +799,10 @@
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B17" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C17" t="s">
         <v>27</v>
@@ -778,10 +810,10 @@
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B18" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C18" t="s">
         <v>27</v>
@@ -789,10 +821,10 @@
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B19" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C19" t="s">
         <v>27</v>
@@ -800,24 +832,21 @@
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B20" t="s">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="C20" t="s">
-        <v>36</v>
-      </c>
-      <c r="D20" t="s">
-        <v>38</v>
+        <v>27</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B21" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C21" t="s">
         <v>27</v>
@@ -825,46 +854,49 @@
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B22" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C22" t="s">
-        <v>36</v>
-      </c>
-      <c r="D22" t="s">
-        <v>39</v>
+        <v>27</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="B23" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="C23" t="s">
         <v>27</v>
+      </c>
+      <c r="D23" t="s">
+        <v>34</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="B24" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C24" t="s">
         <v>27</v>
+      </c>
+      <c r="D24" t="s">
+        <v>34</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="B25" t="s">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="C25" t="s">
         <v>27</v>
@@ -872,52 +904,43 @@
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="B26" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C26" t="s">
-        <v>36</v>
-      </c>
-      <c r="D26" t="s">
-        <v>44</v>
+        <v>27</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="B27" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C27" t="s">
-        <v>36</v>
-      </c>
-      <c r="D27" t="s">
-        <v>40</v>
+        <v>27</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="B28" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C28" t="s">
-        <v>36</v>
-      </c>
-      <c r="D28" t="s">
-        <v>40</v>
+        <v>27</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="B29" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C29" t="s">
         <v>27</v>
@@ -925,27 +948,27 @@
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="B30" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C30" t="s">
-        <v>36</v>
-      </c>
-      <c r="D30" t="s">
-        <v>40</v>
+        <v>27</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B31" t="s">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="C31" t="s">
-        <v>27</v>
+        <v>28</v>
+      </c>
+      <c r="D31" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.3">
@@ -953,10 +976,13 @@
         <v>12</v>
       </c>
       <c r="B32" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C32" t="s">
         <v>28</v>
+      </c>
+      <c r="D32" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.3">
@@ -964,10 +990,13 @@
         <v>12</v>
       </c>
       <c r="B33" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C33" t="s">
         <v>28</v>
+      </c>
+      <c r="D33" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.3">
@@ -975,10 +1004,13 @@
         <v>12</v>
       </c>
       <c r="B34" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C34" t="s">
         <v>28</v>
+      </c>
+      <c r="D34" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.3">
@@ -986,10 +1018,13 @@
         <v>12</v>
       </c>
       <c r="B35" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C35" t="s">
         <v>28</v>
+      </c>
+      <c r="D35" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.3">
@@ -997,15 +1032,18 @@
         <v>12</v>
       </c>
       <c r="B36" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C36" t="s">
         <v>28</v>
+      </c>
+      <c r="D36" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B37" t="s">
         <v>8</v>
@@ -1013,52 +1051,61 @@
       <c r="C37" t="s">
         <v>28</v>
       </c>
+      <c r="D37" t="s">
+        <v>40</v>
+      </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B38" t="s">
         <v>3</v>
       </c>
       <c r="C38" t="s">
-        <v>27</v>
+        <v>28</v>
+      </c>
+      <c r="D38" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B39" t="s">
         <v>4</v>
       </c>
       <c r="C39" t="s">
-        <v>27</v>
+        <v>28</v>
+      </c>
+      <c r="D39" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B40" t="s">
         <v>5</v>
       </c>
       <c r="C40" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D40" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B41" t="s">
         <v>6</v>
       </c>
       <c r="C41" t="s">
-        <v>36</v>
+        <v>28</v>
       </c>
       <c r="D41" t="s">
         <v>40</v>
@@ -1066,13 +1113,13 @@
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B42" t="s">
         <v>7</v>
       </c>
       <c r="C42" t="s">
-        <v>36</v>
+        <v>28</v>
       </c>
       <c r="D42" t="s">
         <v>40</v>
@@ -1080,13 +1127,16 @@
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B43" t="s">
         <v>8</v>
       </c>
       <c r="C43" t="s">
         <v>28</v>
+      </c>
+      <c r="D43" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.3">
@@ -1094,10 +1144,13 @@
         <v>14</v>
       </c>
       <c r="B44" t="s">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="C44" t="s">
         <v>28</v>
+      </c>
+      <c r="D44" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.3">
@@ -1105,10 +1158,13 @@
         <v>14</v>
       </c>
       <c r="B45" t="s">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="C45" t="s">
         <v>28</v>
+      </c>
+      <c r="D45" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.3">
@@ -1116,10 +1172,13 @@
         <v>14</v>
       </c>
       <c r="B46" t="s">
-        <v>5</v>
+        <v>17</v>
       </c>
       <c r="C46" t="s">
         <v>28</v>
+      </c>
+      <c r="D46" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.3">
@@ -1127,10 +1186,13 @@
         <v>14</v>
       </c>
       <c r="B47" t="s">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="C47" t="s">
         <v>28</v>
+      </c>
+      <c r="D47" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.3">
@@ -1138,10 +1200,13 @@
         <v>14</v>
       </c>
       <c r="B48" t="s">
-        <v>7</v>
+        <v>19</v>
       </c>
       <c r="C48" t="s">
         <v>28</v>
+      </c>
+      <c r="D48" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.3">
@@ -1149,73 +1214,91 @@
         <v>14</v>
       </c>
       <c r="B49" t="s">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="C49" t="s">
         <v>28</v>
+      </c>
+      <c r="D49" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="B50" t="s">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="C50" t="s">
         <v>28</v>
+      </c>
+      <c r="D50" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="B51" t="s">
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="C51" t="s">
         <v>28</v>
+      </c>
+      <c r="D51" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="B52" t="s">
-        <v>17</v>
+        <v>6</v>
       </c>
       <c r="C52" t="s">
         <v>28</v>
+      </c>
+      <c r="D52" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="B53" t="s">
-        <v>18</v>
+        <v>7</v>
       </c>
       <c r="C53" t="s">
         <v>28</v>
+      </c>
+      <c r="D53" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="B54" t="s">
-        <v>19</v>
+        <v>8</v>
       </c>
       <c r="C54" t="s">
         <v>28</v>
+      </c>
+      <c r="D54" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="B55" t="s">
-        <v>20</v>
+        <v>3</v>
       </c>
       <c r="C55" t="s">
         <v>28</v>
@@ -1223,30 +1306,24 @@
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B56" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C56" t="s">
-        <v>27</v>
-      </c>
-      <c r="D56" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B57" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C57" t="s">
-        <v>27</v>
-      </c>
-      <c r="D57" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.3">
@@ -1257,73 +1334,94 @@
         <v>3</v>
       </c>
       <c r="C58" t="s">
-        <v>42</v>
+        <v>38</v>
+      </c>
+      <c r="D58" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
-        <v>22</v>
+        <v>2</v>
       </c>
       <c r="B59" t="s">
         <v>4</v>
       </c>
       <c r="C59" t="s">
-        <v>28</v>
+        <v>29</v>
+      </c>
+      <c r="D59" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
-        <v>22</v>
+        <v>2</v>
       </c>
       <c r="B60" t="s">
         <v>5</v>
       </c>
       <c r="C60" t="s">
-        <v>28</v>
+        <v>29</v>
+      </c>
+      <c r="D60" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
-        <v>22</v>
+        <v>2</v>
       </c>
       <c r="B61" t="s">
         <v>6</v>
       </c>
       <c r="C61" t="s">
-        <v>28</v>
+        <v>29</v>
+      </c>
+      <c r="D61" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
-        <v>22</v>
+        <v>2</v>
       </c>
       <c r="B62" t="s">
         <v>7</v>
       </c>
       <c r="C62" t="s">
-        <v>28</v>
+        <v>29</v>
+      </c>
+      <c r="D62" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
-        <v>22</v>
+        <v>2</v>
       </c>
       <c r="B63" t="s">
         <v>8</v>
       </c>
       <c r="C63" t="s">
-        <v>28</v>
+        <v>29</v>
+      </c>
+      <c r="D63" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="B64" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C64" t="s">
-        <v>28</v>
+        <v>29</v>
+      </c>
+      <c r="D64" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.3">
@@ -1331,101 +1429,125 @@
         <v>23</v>
       </c>
       <c r="B65" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C65" t="s">
-        <v>28</v>
+        <v>29</v>
+      </c>
+      <c r="D65" s="2" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
-        <v>23</v>
+        <v>10</v>
       </c>
       <c r="B66" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C66" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="D66" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
-        <v>23</v>
+        <v>10</v>
       </c>
       <c r="B67" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C67" t="s">
-        <v>28</v>
+        <v>35</v>
+      </c>
+      <c r="D67" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
-        <v>25</v>
+        <v>11</v>
       </c>
       <c r="B68" t="s">
         <v>3</v>
       </c>
       <c r="C68" t="s">
-        <v>27</v>
+        <v>35</v>
+      </c>
+      <c r="D68" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
-        <v>25</v>
+        <v>11</v>
       </c>
       <c r="B69" t="s">
         <v>4</v>
       </c>
       <c r="C69" t="s">
-        <v>27</v>
+        <v>35</v>
+      </c>
+      <c r="D69" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
-        <v>25</v>
+        <v>11</v>
       </c>
       <c r="B70" t="s">
         <v>5</v>
       </c>
       <c r="C70" t="s">
-        <v>27</v>
+        <v>35</v>
+      </c>
+      <c r="D70" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
-        <v>25</v>
+        <v>11</v>
       </c>
       <c r="B71" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C71" t="s">
-        <v>27</v>
+        <v>35</v>
+      </c>
+      <c r="D71" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="B72" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C72" t="s">
-        <v>27</v>
+        <v>35</v>
+      </c>
+      <c r="D72" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="B73" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C73" t="s">
-        <v>27</v>
+        <v>35</v>
+      </c>
+      <c r="D73" t="s">
+        <v>47</v>
       </c>
     </row>
   </sheetData>
@@ -1434,4 +1556,1006 @@
     <tablePart r:id="rId1"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{060ACA38-57A0-4FC9-B0DF-07BCFF29244E}">
+  <dimension ref="A1:I73"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="18.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="20.88671875" customWidth="1"/>
+    <col min="6" max="6" width="24.21875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="27.44140625" customWidth="1"/>
+    <col min="8" max="8" width="15.6640625" customWidth="1"/>
+    <col min="9" max="9" width="34.21875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D1" t="s">
+        <v>33</v>
+      </c>
+      <c r="E1" t="s">
+        <v>48</v>
+      </c>
+      <c r="F1" t="s">
+        <v>49</v>
+      </c>
+      <c r="G1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" t="s">
+        <v>27</v>
+      </c>
+      <c r="H2" t="s">
+        <v>27</v>
+      </c>
+      <c r="I2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C3" t="s">
+        <v>27</v>
+      </c>
+      <c r="H3" t="s">
+        <v>28</v>
+      </c>
+      <c r="I3" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B4" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" t="s">
+        <v>27</v>
+      </c>
+      <c r="H4" t="s">
+        <v>29</v>
+      </c>
+      <c r="I4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>24</v>
+      </c>
+      <c r="B5" t="s">
+        <v>6</v>
+      </c>
+      <c r="C5" t="s">
+        <v>27</v>
+      </c>
+      <c r="H5" t="s">
+        <v>35</v>
+      </c>
+      <c r="I5" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>24</v>
+      </c>
+      <c r="B6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C6" t="s">
+        <v>27</v>
+      </c>
+      <c r="F6" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>24</v>
+      </c>
+      <c r="B7" t="s">
+        <v>8</v>
+      </c>
+      <c r="C7" t="s">
+        <v>27</v>
+      </c>
+      <c r="F7" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>2</v>
+      </c>
+      <c r="B8" t="s">
+        <v>3</v>
+      </c>
+      <c r="C8" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9" t="s">
+        <v>3</v>
+      </c>
+      <c r="C9" t="s">
+        <v>27</v>
+      </c>
+      <c r="D9" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
+        <v>4</v>
+      </c>
+      <c r="C10" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>9</v>
+      </c>
+      <c r="B11" t="s">
+        <v>5</v>
+      </c>
+      <c r="C11" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>9</v>
+      </c>
+      <c r="B12" t="s">
+        <v>6</v>
+      </c>
+      <c r="C12" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>9</v>
+      </c>
+      <c r="B13" t="s">
+        <v>7</v>
+      </c>
+      <c r="C13" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>9</v>
+      </c>
+      <c r="B14" t="s">
+        <v>8</v>
+      </c>
+      <c r="C14" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>10</v>
+      </c>
+      <c r="B15" t="s">
+        <v>4</v>
+      </c>
+      <c r="C15" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>10</v>
+      </c>
+      <c r="B16" t="s">
+        <v>6</v>
+      </c>
+      <c r="C16" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>10</v>
+      </c>
+      <c r="B17" t="s">
+        <v>7</v>
+      </c>
+      <c r="C17" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>10</v>
+      </c>
+      <c r="B18" t="s">
+        <v>8</v>
+      </c>
+      <c r="C18" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>11</v>
+      </c>
+      <c r="B19" t="s">
+        <v>6</v>
+      </c>
+      <c r="C19" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>11</v>
+      </c>
+      <c r="B20" t="s">
+        <v>8</v>
+      </c>
+      <c r="C20" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>13</v>
+      </c>
+      <c r="B21" t="s">
+        <v>3</v>
+      </c>
+      <c r="C21" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>13</v>
+      </c>
+      <c r="B22" t="s">
+        <v>4</v>
+      </c>
+      <c r="C22" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>21</v>
+      </c>
+      <c r="B23" t="s">
+        <v>3</v>
+      </c>
+      <c r="C23" t="s">
+        <v>27</v>
+      </c>
+      <c r="D23" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>21</v>
+      </c>
+      <c r="B24" t="s">
+        <v>4</v>
+      </c>
+      <c r="C24" t="s">
+        <v>27</v>
+      </c>
+      <c r="D24" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>25</v>
+      </c>
+      <c r="B25" t="s">
+        <v>3</v>
+      </c>
+      <c r="C25" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>25</v>
+      </c>
+      <c r="B26" t="s">
+        <v>4</v>
+      </c>
+      <c r="C26" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>25</v>
+      </c>
+      <c r="B27" t="s">
+        <v>5</v>
+      </c>
+      <c r="C27" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>25</v>
+      </c>
+      <c r="B28" t="s">
+        <v>6</v>
+      </c>
+      <c r="C28" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
+        <v>25</v>
+      </c>
+      <c r="B29" t="s">
+        <v>7</v>
+      </c>
+      <c r="C29" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
+        <v>25</v>
+      </c>
+      <c r="B30" t="s">
+        <v>8</v>
+      </c>
+      <c r="C30" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>12</v>
+      </c>
+      <c r="B31" t="s">
+        <v>3</v>
+      </c>
+      <c r="C31" t="s">
+        <v>28</v>
+      </c>
+      <c r="D31" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
+        <v>12</v>
+      </c>
+      <c r="B32" t="s">
+        <v>4</v>
+      </c>
+      <c r="C32" t="s">
+        <v>28</v>
+      </c>
+      <c r="D32" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
+        <v>12</v>
+      </c>
+      <c r="B33" t="s">
+        <v>5</v>
+      </c>
+      <c r="C33" t="s">
+        <v>28</v>
+      </c>
+      <c r="D33" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A34" t="s">
+        <v>12</v>
+      </c>
+      <c r="B34" t="s">
+        <v>6</v>
+      </c>
+      <c r="C34" t="s">
+        <v>28</v>
+      </c>
+      <c r="D34" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
+        <v>12</v>
+      </c>
+      <c r="B35" t="s">
+        <v>7</v>
+      </c>
+      <c r="C35" t="s">
+        <v>28</v>
+      </c>
+      <c r="D35" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A36" t="s">
+        <v>12</v>
+      </c>
+      <c r="B36" t="s">
+        <v>8</v>
+      </c>
+      <c r="C36" t="s">
+        <v>28</v>
+      </c>
+      <c r="D36" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A37" t="s">
+        <v>13</v>
+      </c>
+      <c r="B37" t="s">
+        <v>8</v>
+      </c>
+      <c r="C37" t="s">
+        <v>28</v>
+      </c>
+      <c r="D37" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A38" t="s">
+        <v>14</v>
+      </c>
+      <c r="B38" t="s">
+        <v>3</v>
+      </c>
+      <c r="C38" t="s">
+        <v>28</v>
+      </c>
+      <c r="D38" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A39" t="s">
+        <v>14</v>
+      </c>
+      <c r="B39" t="s">
+        <v>4</v>
+      </c>
+      <c r="C39" t="s">
+        <v>28</v>
+      </c>
+      <c r="D39" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A40" t="s">
+        <v>14</v>
+      </c>
+      <c r="B40" t="s">
+        <v>5</v>
+      </c>
+      <c r="C40" t="s">
+        <v>28</v>
+      </c>
+      <c r="D40" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A41" t="s">
+        <v>14</v>
+      </c>
+      <c r="B41" t="s">
+        <v>6</v>
+      </c>
+      <c r="C41" t="s">
+        <v>28</v>
+      </c>
+      <c r="D41" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A42" t="s">
+        <v>14</v>
+      </c>
+      <c r="B42" t="s">
+        <v>7</v>
+      </c>
+      <c r="C42" t="s">
+        <v>28</v>
+      </c>
+      <c r="D42" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A43" t="s">
+        <v>14</v>
+      </c>
+      <c r="B43" t="s">
+        <v>8</v>
+      </c>
+      <c r="C43" t="s">
+        <v>28</v>
+      </c>
+      <c r="D43" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A44" t="s">
+        <v>14</v>
+      </c>
+      <c r="B44" t="s">
+        <v>15</v>
+      </c>
+      <c r="C44" t="s">
+        <v>28</v>
+      </c>
+      <c r="D44" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A45" t="s">
+        <v>14</v>
+      </c>
+      <c r="B45" t="s">
+        <v>16</v>
+      </c>
+      <c r="C45" t="s">
+        <v>28</v>
+      </c>
+      <c r="D45" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A46" t="s">
+        <v>14</v>
+      </c>
+      <c r="B46" t="s">
+        <v>17</v>
+      </c>
+      <c r="C46" t="s">
+        <v>28</v>
+      </c>
+      <c r="D46" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A47" t="s">
+        <v>14</v>
+      </c>
+      <c r="B47" t="s">
+        <v>18</v>
+      </c>
+      <c r="C47" t="s">
+        <v>28</v>
+      </c>
+      <c r="D47" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A48" t="s">
+        <v>14</v>
+      </c>
+      <c r="B48" t="s">
+        <v>19</v>
+      </c>
+      <c r="C48" t="s">
+        <v>28</v>
+      </c>
+      <c r="D48" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A49" t="s">
+        <v>14</v>
+      </c>
+      <c r="B49" t="s">
+        <v>20</v>
+      </c>
+      <c r="C49" t="s">
+        <v>28</v>
+      </c>
+      <c r="D49" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A50" t="s">
+        <v>22</v>
+      </c>
+      <c r="B50" t="s">
+        <v>4</v>
+      </c>
+      <c r="C50" t="s">
+        <v>28</v>
+      </c>
+      <c r="D50" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A51" t="s">
+        <v>22</v>
+      </c>
+      <c r="B51" t="s">
+        <v>5</v>
+      </c>
+      <c r="C51" t="s">
+        <v>28</v>
+      </c>
+      <c r="D51" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A52" t="s">
+        <v>22</v>
+      </c>
+      <c r="B52" t="s">
+        <v>6</v>
+      </c>
+      <c r="C52" t="s">
+        <v>28</v>
+      </c>
+      <c r="D52" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A53" t="s">
+        <v>22</v>
+      </c>
+      <c r="B53" t="s">
+        <v>7</v>
+      </c>
+      <c r="C53" t="s">
+        <v>28</v>
+      </c>
+      <c r="D53" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A54" t="s">
+        <v>22</v>
+      </c>
+      <c r="B54" t="s">
+        <v>8</v>
+      </c>
+      <c r="C54" t="s">
+        <v>28</v>
+      </c>
+      <c r="D54" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A55" t="s">
+        <v>23</v>
+      </c>
+      <c r="B55" t="s">
+        <v>3</v>
+      </c>
+      <c r="C55" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A56" t="s">
+        <v>23</v>
+      </c>
+      <c r="B56" t="s">
+        <v>4</v>
+      </c>
+      <c r="C56" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A57" t="s">
+        <v>23</v>
+      </c>
+      <c r="B57" t="s">
+        <v>6</v>
+      </c>
+      <c r="C57" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A58" t="s">
+        <v>22</v>
+      </c>
+      <c r="B58" t="s">
+        <v>3</v>
+      </c>
+      <c r="C58" t="s">
+        <v>38</v>
+      </c>
+      <c r="D58" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A59" t="s">
+        <v>2</v>
+      </c>
+      <c r="B59" t="s">
+        <v>4</v>
+      </c>
+      <c r="C59" t="s">
+        <v>29</v>
+      </c>
+      <c r="D59" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A60" t="s">
+        <v>2</v>
+      </c>
+      <c r="B60" t="s">
+        <v>5</v>
+      </c>
+      <c r="C60" t="s">
+        <v>29</v>
+      </c>
+      <c r="D60" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A61" t="s">
+        <v>2</v>
+      </c>
+      <c r="B61" t="s">
+        <v>6</v>
+      </c>
+      <c r="C61" t="s">
+        <v>29</v>
+      </c>
+      <c r="D61" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A62" t="s">
+        <v>2</v>
+      </c>
+      <c r="B62" t="s">
+        <v>7</v>
+      </c>
+      <c r="C62" t="s">
+        <v>29</v>
+      </c>
+      <c r="D62" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A63" t="s">
+        <v>2</v>
+      </c>
+      <c r="B63" t="s">
+        <v>8</v>
+      </c>
+      <c r="C63" t="s">
+        <v>29</v>
+      </c>
+      <c r="D63" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A64" t="s">
+        <v>13</v>
+      </c>
+      <c r="B64" t="s">
+        <v>5</v>
+      </c>
+      <c r="C64" t="s">
+        <v>29</v>
+      </c>
+      <c r="D64" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A65" t="s">
+        <v>23</v>
+      </c>
+      <c r="B65" t="s">
+        <v>5</v>
+      </c>
+      <c r="C65" t="s">
+        <v>29</v>
+      </c>
+      <c r="D65" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="E65" s="2"/>
+      <c r="F65" s="2"/>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A66" t="s">
+        <v>10</v>
+      </c>
+      <c r="B66" t="s">
+        <v>3</v>
+      </c>
+      <c r="C66" t="s">
+        <v>35</v>
+      </c>
+      <c r="D66" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A67" t="s">
+        <v>10</v>
+      </c>
+      <c r="B67" t="s">
+        <v>5</v>
+      </c>
+      <c r="C67" t="s">
+        <v>35</v>
+      </c>
+      <c r="D67" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A68" t="s">
+        <v>11</v>
+      </c>
+      <c r="B68" t="s">
+        <v>3</v>
+      </c>
+      <c r="C68" t="s">
+        <v>35</v>
+      </c>
+      <c r="D68" t="s">
+        <v>46</v>
+      </c>
+      <c r="F68" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A69" t="s">
+        <v>11</v>
+      </c>
+      <c r="B69" t="s">
+        <v>4</v>
+      </c>
+      <c r="C69" t="s">
+        <v>35</v>
+      </c>
+      <c r="D69" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A70" t="s">
+        <v>11</v>
+      </c>
+      <c r="B70" t="s">
+        <v>5</v>
+      </c>
+      <c r="C70" t="s">
+        <v>35</v>
+      </c>
+      <c r="D70" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A71" t="s">
+        <v>11</v>
+      </c>
+      <c r="B71" t="s">
+        <v>7</v>
+      </c>
+      <c r="C71" t="s">
+        <v>35</v>
+      </c>
+      <c r="D71" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A72" t="s">
+        <v>13</v>
+      </c>
+      <c r="B72" t="s">
+        <v>6</v>
+      </c>
+      <c r="C72" t="s">
+        <v>35</v>
+      </c>
+      <c r="D72" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A73" t="s">
+        <v>13</v>
+      </c>
+      <c r="B73" t="s">
+        <v>7</v>
+      </c>
+      <c r="C73" t="s">
+        <v>35</v>
+      </c>
+      <c r="D73" t="s">
+        <v>47</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
 </file>
</xml_diff>